<commit_message>
added slides for chapter 4 of circuits class, and my lab 1 excel sheet.
</commit_message>
<xml_diff>
--- a/Study_Plans/DcAcCircuits/LAB1.xlsx
+++ b/Study_Plans/DcAcCircuits/LAB1.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esmos\local_Documents\M_Arch\Study_Plans\DcAcCircuits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9BF7972-4BCC-4AF7-A269-F33F4F75BFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB19972D-135D-4C7C-9606-DB9BC570314D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{9790BB06-835B-421B-B574-695F61F1FFC5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{9790BB06-835B-421B-B574-695F61F1FFC5}"/>
   </bookViews>
   <sheets>
     <sheet name="Resistor as X element" sheetId="2" r:id="rId1"/>
     <sheet name="Light Bulb as X element" sheetId="3" r:id="rId2"/>
-    <sheet name="Lab 1 Data" sheetId="1" r:id="rId3"/>
+    <sheet name="Diode as X Element" sheetId="5" r:id="rId3"/>
+    <sheet name="Lab 1 Data" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
   <si>
     <t>DC/AC Circuits Fall 26 Lab 1</t>
   </si>
@@ -70,6 +71,23 @@
   </si>
   <si>
     <t>Light Bulb as X element</t>
+  </si>
+  <si>
+    <r>
+      <t>Diode as X element with R=21.9k</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Ω</t>
+    </r>
+  </si>
+  <si>
+    <t>Diode as X element with R=21.9kΩ</t>
   </si>
 </sst>
 </file>
@@ -111,12 +129,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1178,6 +1195,842 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Diode as Element</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> X</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Positive Diode Voltage</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Lab 1 Data'!$K$7:$K$40</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>10.5</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>11.5</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>12.5</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>13.5</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>14.5</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>15.5</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>16.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Lab 1 Data'!$L$7:$L$40</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.4999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.06</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.11</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.13</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.22</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.24</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.26</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.28000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.3</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.33</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.35</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.37</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.39500000000000002</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.42</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.44</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.46500000000000002</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.49</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.51</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.53</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.55000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.57499999999999996</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.64</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.66</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.69</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.7</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9B2D-4C63-80A2-C1C5C213D884}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Negative Diode Voltage</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="movingAvg"/>
+            <c:period val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Lab 1 Data'!$P$7:$P$40</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-1.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-2.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-3.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-4.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-5.5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-6.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-7</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-7.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-8</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-8.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-9</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-9.5</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>-10</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>-10.5</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>-11</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-11.5</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>-12</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-12.5</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-13</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>-13.5</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>-14</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>-14.5</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>-15</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>-15.5</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>-16</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>-16.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Lab 1 Data'!$Q$7:$Q$40</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="34"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>-0.01</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-0.03</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-0.06</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>-0.08</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>-0.1</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>-0.12</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>-0.15</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>-0.17</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>-0.19</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>-0.21</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-9B2D-4C63-80A2-C1C5C213D884}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1301259808"/>
+        <c:axId val="1871179792"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1301259808"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1871179792"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1871179792"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1301259808"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1258,6 +2111,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1775,6 +2668,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2304,6 +3713,15 @@
   <sheetPr/>
   <pageMargins left="0" right="0" top="0.25" bottom="0.25" header="0" footer="0"/>
   <pageSetup orientation="landscape" blackAndWhite="1" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</chartsheet>
+</file>
+
+<file path=xl/chartsheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{CA01CA76-1F73-4521-AD3D-95567023ECD8}">
+  <sheetPr/>
+  <pageMargins left="0" right="0" top="0.25" bottom="0.25" header="0" footer="0"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </chartsheet>
 </file>
@@ -2352,6 +3770,39 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A5DEBEF-8AEF-9228-D56B-A459FC6EDEB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="9635908" cy="7208990"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00A39E2E-7D27-71C0-E04C-C1D872F464C2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2977,10 +4428,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB76CB45-7837-4F51-AA01-DA599AE307E0}">
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:T40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2999,7 +4450,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -3011,7 +4462,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -3024,8 +4475,17 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
+      <c r="K5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="P5" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -3042,568 +4502,910 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
+      <c r="K6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="P6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>-1.6E-2</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <f>K7*$T$7</f>
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>-1</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.5</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8">
         <v>1.6E-2</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
       <c r="F8">
         <v>0.5</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8">
         <v>8.0299999999999994</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="K8">
+        <v>0.5</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <f t="shared" ref="P8:P40" si="0">K8*$T$7</f>
+        <v>-0.5</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
       <c r="F9">
         <v>1</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9">
         <v>10.3</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1.5</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
       <c r="F10">
         <v>1.5</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10">
         <v>12.07</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="K10">
+        <v>1.5</v>
+      </c>
+      <c r="L10">
+        <v>0.04</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="0"/>
+        <v>-1.5</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11">
         <v>0.06</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
       <c r="F11">
         <v>2</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11">
         <v>14.22</v>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="K11">
+        <v>2</v>
+      </c>
+      <c r="L11">
+        <v>0.06</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="0"/>
+        <v>-2</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2.5</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12">
         <v>7.5999999999999998E-2</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
       <c r="F12">
         <v>2.5</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12">
         <v>16.12</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="K12">
+        <v>2.5</v>
+      </c>
+      <c r="L12">
+        <v>0.08</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="0"/>
+        <v>-2.5</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>3</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
       <c r="F13">
         <v>3</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13">
         <v>17.73</v>
       </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="K13">
+        <v>3</v>
+      </c>
+      <c r="L13">
+        <v>0.11</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="0"/>
+        <v>-3</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3.5</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14">
         <v>0.107</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
       <c r="F14">
         <v>3.5</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14">
         <v>19.55</v>
       </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="K14">
+        <v>3.5</v>
+      </c>
+      <c r="L14">
+        <v>0.13</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="0"/>
+        <v>-3.5</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15">
         <v>0.12</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
       <c r="F15">
         <v>4</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15">
         <v>20.91</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="K15">
+        <v>4</v>
+      </c>
+      <c r="L15">
+        <v>0.15</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="0"/>
+        <v>-4</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>4.5</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16">
         <v>0.13700000000000001</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
       <c r="F16">
         <v>4.5</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16">
         <v>22.63</v>
       </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="K16">
+        <v>4.5</v>
+      </c>
+      <c r="L16">
+        <v>0.17</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="0"/>
+        <v>-4.5</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>5</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17">
         <v>0.151</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
       <c r="F17">
         <v>5</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17">
         <v>24.06</v>
       </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="K17">
+        <v>5</v>
+      </c>
+      <c r="L17">
+        <v>0.19</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="0"/>
+        <v>-5</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>5.5</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18">
         <v>0.16800000000000001</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
       <c r="F18">
         <v>5.5</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18">
         <v>25.43</v>
       </c>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="K18">
+        <v>5.5</v>
+      </c>
+      <c r="L18">
+        <v>0.22</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="0"/>
+        <v>-5.5</v>
+      </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>6</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19">
         <v>0.18099999999999999</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
       <c r="F19">
         <v>6</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19">
         <v>26.73</v>
       </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
+      <c r="K19">
+        <v>6</v>
+      </c>
+      <c r="L19">
+        <v>0.24</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="0"/>
+        <v>-6</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>6.5</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20">
         <v>0.19800000000000001</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
       <c r="F20">
         <v>6.5</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20">
         <v>28.06</v>
       </c>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
+      <c r="K20">
+        <v>6.5</v>
+      </c>
+      <c r="L20">
+        <v>0.26</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="0"/>
+        <v>-6.5</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>7</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21">
         <v>0.21199999999999999</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
       <c r="F21">
         <v>7</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21">
         <v>29.36</v>
       </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
+      <c r="K21">
+        <v>7</v>
+      </c>
+      <c r="L21">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="0"/>
+        <v>-7</v>
+      </c>
+      <c r="Q21">
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>7.5</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22">
         <v>0.22500000000000001</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
       <c r="F22">
         <v>7.5</v>
       </c>
-      <c r="G22" s="2">
+      <c r="G22">
         <v>30.53</v>
       </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
+      <c r="K22">
+        <v>7.5</v>
+      </c>
+      <c r="L22">
+        <v>0.3</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="0"/>
+        <v>-7.5</v>
+      </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>8</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23">
         <v>0.24299999999999999</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
       <c r="F23">
         <v>8</v>
       </c>
-      <c r="G23" s="2">
+      <c r="G23">
         <v>31.74</v>
       </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+      <c r="K23">
+        <v>8</v>
+      </c>
+      <c r="L23">
+        <v>0.33</v>
+      </c>
+      <c r="P23">
+        <f t="shared" si="0"/>
+        <v>-8</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>8.5</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24">
         <v>0.25600000000000001</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
       <c r="F24">
         <v>8.5</v>
       </c>
-      <c r="G24" s="2">
+      <c r="G24">
         <v>32.880000000000003</v>
       </c>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
+      <c r="K24">
+        <v>8.5</v>
+      </c>
+      <c r="L24">
+        <v>0.35</v>
+      </c>
+      <c r="P24">
+        <f t="shared" si="0"/>
+        <v>-8.5</v>
+      </c>
+      <c r="Q24">
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>9</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25">
         <v>0.27200000000000002</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
       <c r="F25">
         <v>9</v>
       </c>
-      <c r="G25" s="2">
+      <c r="G25">
         <v>33.97</v>
       </c>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
+      <c r="K25">
+        <v>9</v>
+      </c>
+      <c r="L25">
+        <v>0.37</v>
+      </c>
+      <c r="P25">
+        <f t="shared" si="0"/>
+        <v>-9</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>9.5</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26">
         <v>0.28499999999999998</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
       <c r="F26">
         <v>9.5</v>
       </c>
-      <c r="G26" s="2">
+      <c r="G26">
         <v>35.130000000000003</v>
       </c>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
+      <c r="K26">
+        <v>9.5</v>
+      </c>
+      <c r="L26">
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="P26">
+        <f t="shared" si="0"/>
+        <v>-9.5</v>
+      </c>
+      <c r="Q26">
+        <v>0</v>
+      </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>10</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27">
         <v>0.30099999999999999</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
       <c r="F27">
         <v>10</v>
       </c>
-      <c r="G27" s="2">
+      <c r="G27">
         <v>36.090000000000003</v>
       </c>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
+      <c r="K27">
+        <v>10</v>
+      </c>
+      <c r="L27">
+        <v>0.42</v>
+      </c>
+      <c r="P27">
+        <f t="shared" si="0"/>
+        <v>-10</v>
+      </c>
+      <c r="Q27">
+        <v>0</v>
+      </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>10.5</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28">
         <v>0.315</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
       <c r="F28">
         <v>10.5</v>
       </c>
-      <c r="G28" s="2">
+      <c r="G28">
         <v>37.020000000000003</v>
       </c>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
+      <c r="K28">
+        <v>10.5</v>
+      </c>
+      <c r="L28">
+        <v>0.44</v>
+      </c>
+      <c r="P28">
+        <f t="shared" si="0"/>
+        <v>-10.5</v>
+      </c>
+      <c r="Q28">
+        <v>0</v>
+      </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>11</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29">
         <v>0.33</v>
       </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
       <c r="F29">
         <v>11</v>
       </c>
-      <c r="G29" s="2">
+      <c r="G29">
         <v>38.08</v>
       </c>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
+      <c r="K29">
+        <v>11</v>
+      </c>
+      <c r="L29">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="P29">
+        <f t="shared" si="0"/>
+        <v>-11</v>
+      </c>
+      <c r="Q29">
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>11.5</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30">
         <v>0.34499999999999997</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
       <c r="F30">
         <v>11.5</v>
       </c>
-      <c r="G30" s="2">
+      <c r="G30">
         <v>39.15</v>
       </c>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
+      <c r="K30">
+        <v>11.5</v>
+      </c>
+      <c r="L30">
+        <v>0.49</v>
+      </c>
+      <c r="P30">
+        <f t="shared" si="0"/>
+        <v>-11.5</v>
+      </c>
+      <c r="Q30">
+        <v>0</v>
+      </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>12</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31">
         <v>0.36299999999999999</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
       <c r="F31">
         <v>12</v>
       </c>
-      <c r="G31" s="2">
+      <c r="G31">
         <v>40.25</v>
       </c>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
+      <c r="K31">
+        <v>12</v>
+      </c>
+      <c r="L31">
+        <v>0.51</v>
+      </c>
+      <c r="P31">
+        <f t="shared" si="0"/>
+        <v>-12</v>
+      </c>
+      <c r="Q31">
+        <v>-0.01</v>
+      </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>12.5</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32">
         <v>0.376</v>
       </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
       <c r="F32">
         <v>12.5</v>
       </c>
-      <c r="G32" s="2">
+      <c r="G32">
         <v>41.27</v>
       </c>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
+      <c r="K32">
+        <v>12.5</v>
+      </c>
+      <c r="L32">
+        <v>0.53</v>
+      </c>
+      <c r="P32">
+        <f t="shared" si="0"/>
+        <v>-12.5</v>
+      </c>
+      <c r="Q32">
+        <v>-0.03</v>
+      </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>13</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33">
         <v>0.39200000000000002</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
       <c r="F33">
         <v>13</v>
       </c>
-      <c r="G33" s="2">
+      <c r="G33">
         <v>42.33</v>
       </c>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
+      <c r="K33">
+        <v>13</v>
+      </c>
+      <c r="L33">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="P33">
+        <f t="shared" si="0"/>
+        <v>-13</v>
+      </c>
+      <c r="Q33">
+        <v>-0.06</v>
+      </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>13.5</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34">
         <v>0.40699999999999997</v>
       </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
       <c r="F34">
         <v>13.5</v>
       </c>
-      <c r="G34" s="2">
+      <c r="G34">
         <v>43.24</v>
       </c>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
+      <c r="K34">
+        <v>13.5</v>
+      </c>
+      <c r="L34">
+        <v>0.57499999999999996</v>
+      </c>
+      <c r="P34">
+        <f t="shared" si="0"/>
+        <v>-13.5</v>
+      </c>
+      <c r="Q34">
+        <v>-0.08</v>
+      </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>14</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35">
         <v>0.42</v>
       </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
       <c r="F35">
         <v>14</v>
       </c>
-      <c r="G35" s="2">
+      <c r="G35">
         <v>43.66</v>
       </c>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
+      <c r="K35">
+        <v>14</v>
+      </c>
+      <c r="L35">
+        <v>0.6</v>
+      </c>
+      <c r="P35">
+        <f t="shared" si="0"/>
+        <v>-14</v>
+      </c>
+      <c r="Q35">
+        <v>-0.1</v>
+      </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>14.5</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36">
         <v>0.435</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
       <c r="F36">
         <v>14.5</v>
       </c>
-      <c r="G36" s="2">
+      <c r="G36">
         <v>44.72</v>
       </c>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+      <c r="K36">
+        <v>14.5</v>
+      </c>
+      <c r="L36">
+        <v>0.62</v>
+      </c>
+      <c r="P36">
+        <f t="shared" si="0"/>
+        <v>-14.5</v>
+      </c>
+      <c r="Q36">
+        <v>-0.12</v>
+      </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>15</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37">
         <v>0.45100000000000001</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
       <c r="F37">
         <v>15</v>
       </c>
-      <c r="G37" s="2">
+      <c r="G37">
         <v>45.69</v>
       </c>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
+      <c r="K37">
+        <v>15</v>
+      </c>
+      <c r="L37">
+        <v>0.64</v>
+      </c>
+      <c r="P37">
+        <f t="shared" si="0"/>
+        <v>-15</v>
+      </c>
+      <c r="Q37">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K38">
+        <v>15.5</v>
+      </c>
+      <c r="L38">
+        <v>0.66</v>
+      </c>
+      <c r="P38">
+        <f t="shared" si="0"/>
+        <v>-15.5</v>
+      </c>
+      <c r="Q38">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K39">
+        <v>16</v>
+      </c>
+      <c r="L39">
+        <v>0.69</v>
+      </c>
+      <c r="P39">
+        <f t="shared" si="0"/>
+        <v>-16</v>
+      </c>
+      <c r="Q39">
+        <v>-0.19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K40">
+        <v>16.3</v>
+      </c>
+      <c r="L40">
+        <v>0.7</v>
+      </c>
+      <c r="P40">
+        <f t="shared" si="0"/>
+        <v>-16.3</v>
+      </c>
+      <c r="Q40">
+        <v>-0.21</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="F5:I5"/>
     <mergeCell ref="G6:I6"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="K5:N5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>